<commit_message>
Add WhatsApp integration and Twilio dependencies
</commit_message>
<xml_diff>
--- a/PC/Seat Availibility.xlsx
+++ b/PC/Seat Availibility.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mukesh.kumar\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mukesh.kumar\PycharmProjects\pc_vectorless_rag\PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB32E7BB-772D-491C-A503-C75135512FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EB56AE-4BAE-4527-AD77-C72C25AD40BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DC0F0EB2-A80F-4677-ADBA-A213D341B11A}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>Available From</t>
   </si>
   <si>
-    <t>Type of Room</t>
-  </si>
-  <si>
     <t>Rent/Month
 (For &gt; 2 Months)</t>
   </si>
@@ -104,6 +101,9 @@
   </si>
   <si>
     <t>House-Keeping | 24X7 water | Water Coller &amp; Purifier | 24X7 warden | Power Backup | Wi-Fi | Paid Laundry | CCTV | Bio-Matric Entry &amp; Exit</t>
+  </si>
+  <si>
+    <t>Availbale Type of Room</t>
   </si>
 </sst>
 </file>
@@ -651,27 +651,27 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="4">
+        <v>46113</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" s="4">
-        <v>46082</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>7</v>
       </c>
       <c r="D2" s="6">
         <v>3850</v>
@@ -685,13 +685,13 @@
     </row>
     <row r="3" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4">
+        <v>46113</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="4">
-        <v>46082</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="D3" s="6">
         <v>3300</v>
@@ -705,13 +705,13 @@
     </row>
     <row r="4" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="4">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="6">
         <v>3300</v>
@@ -725,13 +725,13 @@
     </row>
     <row r="5" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4">
+        <v>46113</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="B5" s="4">
-        <v>46082</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>12</v>
       </c>
       <c r="D5" s="6">
         <v>4400</v>
@@ -745,13 +745,13 @@
     </row>
     <row r="6" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4">
+        <v>46113</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="B6" s="4">
-        <v>46082</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>14</v>
       </c>
       <c r="D6" s="6">
         <v>4400</v>
@@ -765,13 +765,13 @@
     </row>
     <row r="7" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="4">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" s="6">
         <v>4400</v>
@@ -785,13 +785,13 @@
     </row>
     <row r="8" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="4">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" s="6">
         <v>4400</v>
@@ -813,7 +813,7 @@
     </row>
     <row r="10" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -823,7 +823,7 @@
     </row>
     <row r="11" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -833,7 +833,7 @@
     </row>
     <row r="12" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A12" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -843,7 +843,7 @@
     </row>
     <row r="13" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -853,7 +853,7 @@
     </row>
     <row r="14" spans="1:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>

</xml_diff>